<commit_message>
feat: W20 · Módulo Histórico Reactivo CR + RND · 16 cards interactivas · Mayo 2026
</commit_message>
<xml_diff>
--- a/checkrates/week-20/Analisis_Checkrates_7d.xlsx
+++ b/checkrates/week-20/Analisis_Checkrates_7d.xlsx
@@ -569,7 +569,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 19/05/2026 05:04 · W20 · 12-18 may 2026</t>
+          <t>Generado: 21/05/2026 22:18 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -725,7 +725,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 19/05/2026 05:04 · W20 · 12-18 may 2026</t>
+          <t>Generado: 21/05/2026 22:18 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 19/05/2026 05:04 · W20 · 12-18 may 2026</t>
+          <t>Generado: 21/05/2026 22:18 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1178,7 +1178,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 19/05/2026 05:04 · W20 · 12-18 may 2026</t>
+          <t>Generado: 21/05/2026 22:18 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1338,7 +1338,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 19/05/2026 05:04 · W20 · 12-18 may 2026</t>
+          <t>Generado: 21/05/2026 22:18 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1892,7 +1892,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 19/05/2026 05:04 · W20 · 12-18 may 2026</t>
+          <t>Generado: 21/05/2026 22:18 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -5099,7 +5099,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 19/05/2026 05:04 · W20 · 12-18 may 2026</t>
+          <t>Generado: 21/05/2026 22:18 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -9398,7 +9398,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 19/05/2026 05:04 · W20 · 12-18 may 2026</t>
+          <t>Generado: 21/05/2026 22:18 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -10736,7 +10736,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 19/05/2026 05:04 · W20 · 12-18 may 2026</t>
+          <t>Generado: 21/05/2026 22:18 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -14330,7 +14330,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 19/05/2026 05:04 · W20 · 12-18 may 2026</t>
+          <t>Generado: 21/05/2026 22:18 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -14669,7 +14669,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 19/05/2026 05:04 · W20 · 12-18 may 2026</t>
+          <t>Generado: 21/05/2026 22:18 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -18752,7 +18752,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 19/05/2026 05:04 · W20 · 12-18 may 2026</t>
+          <t>Generado: 21/05/2026 22:18 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -18905,7 +18905,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 19/05/2026 05:04 · W20 · 12-18 may 2026</t>
+          <t>Generado: 21/05/2026 22:18 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -19058,7 +19058,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 19/05/2026 05:04 · W20 · 12-18 may 2026</t>
+          <t>Generado: 21/05/2026 22:18 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -19218,7 +19218,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 19/05/2026 05:04 · W20 · 12-18 may 2026</t>
+          <t>Generado: 21/05/2026 22:18 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -23822,7 +23822,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 19/05/2026 05:04 · W20 · 12-18 may 2026</t>
+          <t>Generado: 21/05/2026 22:18 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -28121,7 +28121,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 19/05/2026 05:04 · W20 · 12-18 may 2026</t>
+          <t>Generado: 21/05/2026 22:18 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -32420,7 +32420,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 19/05/2026 05:04 · W20 · 12-18 may 2026</t>
+          <t>Generado: 21/05/2026 22:18 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -34278,7 +34278,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 19/05/2026 05:04 · W20 · 12-18 may 2026</t>
+          <t>Generado: 21/05/2026 22:18 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -37872,7 +37872,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 19/05/2026 05:04 · W20 · 12-18 may 2026</t>
+          <t>Generado: 21/05/2026 22:18 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -38291,7 +38291,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 19/05/2026 05:04 · W20 · 12-18 may 2026</t>
+          <t>Generado: 21/05/2026 22:18 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -42584,7 +42584,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 19/05/2026 05:04 · W20 · 12-18 may 2026</t>
+          <t>Generado: 21/05/2026 22:18 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -42744,7 +42744,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 19/05/2026 05:04 · W20 · 12-18 may 2026</t>
+          <t>Generado: 21/05/2026 22:18 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -47342,7 +47342,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 19/05/2026 05:04 · W20 · 12-18 may 2026</t>
+          <t>Generado: 21/05/2026 22:18 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -47502,7 +47502,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 19/05/2026 05:04 · W20 · 12-18 may 2026</t>
+          <t>Generado: 21/05/2026 22:18 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -50981,7 +50981,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 19/05/2026 05:04 · W20 · 12-18 may 2026</t>
+          <t>Generado: 21/05/2026 22:18 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -55280,7 +55280,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 19/05/2026 05:04 · W20 · 12-18 may 2026</t>
+          <t>Generado: 21/05/2026 22:18 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -59579,7 +59579,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 19/05/2026 05:04 · W20 · 12-18 may 2026</t>
+          <t>Generado: 21/05/2026 22:18 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -61357,7 +61357,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 19/05/2026 05:04 · W20 · 12-18 may 2026</t>
+          <t>Generado: 21/05/2026 22:18 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -64951,7 +64951,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 19/05/2026 05:04 · W20 · 12-18 may 2026</t>
+          <t>Generado: 21/05/2026 22:18 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -65370,7 +65370,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 19/05/2026 05:04 · W20 · 12-18 may 2026</t>
+          <t>Generado: 21/05/2026 22:18 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -69669,7 +69669,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 19/05/2026 05:04 · W20 · 12-18 may 2026</t>
+          <t>Generado: 21/05/2026 22:18 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -73967,7 +73967,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 19/05/2026 05:04 · W20 · 12-18 may 2026</t>
+          <t>Generado: 21/05/2026 22:18 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -77961,7 +77961,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 19/05/2026 05:04 · W20 · 12-18 may 2026</t>
+          <t>Generado: 21/05/2026 22:18 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -80139,7 +80139,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 19/05/2026 05:04 · W20 · 12-18 may 2026</t>
+          <t>Generado: 21/05/2026 22:18 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -83733,7 +83733,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 19/05/2026 05:04 · W20 · 12-18 may 2026</t>
+          <t>Generado: 21/05/2026 22:18 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -84152,7 +84152,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 19/05/2026 05:04 · W20 · 12-18 may 2026</t>
+          <t>Generado: 21/05/2026 22:18 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Week 20 · RatesNoDispo + CheckRates + hub index · 11–17 may 2026
- Reportes editoriales CR y RND regenerados con fixes UI batch
- Excels actualizados (8 archivos · 33+37 pestañas)
- index.html hub actualizado con KPIs W20
- Mail_W20.html generado
- render_mail_v3.py: fix keys pickle W20 (global_w18→global_w20)
- build_package.py: fix import template_seguimiento + logo_b64
</commit_message>
<xml_diff>
--- a/checkrates/week-20/Analisis_Checkrates_7d.xlsx
+++ b/checkrates/week-20/Analisis_Checkrates_7d.xlsx
@@ -569,7 +569,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 02:24 · W20 · 12-18 may 2026</t>
+          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -725,7 +725,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 02:24 · W20 · 12-18 may 2026</t>
+          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 02:24 · W20 · 12-18 may 2026</t>
+          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1178,7 +1178,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 02:24 · W20 · 12-18 may 2026</t>
+          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1338,7 +1338,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 02:24 · W20 · 12-18 may 2026</t>
+          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1892,7 +1892,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 02:24 · W20 · 12-18 may 2026</t>
+          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -5099,7 +5099,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 02:24 · W20 · 12-18 may 2026</t>
+          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -9398,7 +9398,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 02:24 · W20 · 12-18 may 2026</t>
+          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -10736,7 +10736,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 02:24 · W20 · 12-18 may 2026</t>
+          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -14330,7 +14330,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 02:24 · W20 · 12-18 may 2026</t>
+          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -14669,7 +14669,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 02:24 · W20 · 12-18 may 2026</t>
+          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -18752,7 +18752,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 02:24 · W20 · 12-18 may 2026</t>
+          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -18905,7 +18905,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 02:24 · W20 · 12-18 may 2026</t>
+          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -19058,7 +19058,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 02:24 · W20 · 12-18 may 2026</t>
+          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -19218,7 +19218,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 02:24 · W20 · 12-18 may 2026</t>
+          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -23822,7 +23822,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 02:24 · W20 · 12-18 may 2026</t>
+          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -28121,7 +28121,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 02:24 · W20 · 12-18 may 2026</t>
+          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -32420,7 +32420,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 02:24 · W20 · 12-18 may 2026</t>
+          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -34278,7 +34278,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 02:24 · W20 · 12-18 may 2026</t>
+          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -37872,7 +37872,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 02:24 · W20 · 12-18 may 2026</t>
+          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -38291,7 +38291,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 02:24 · W20 · 12-18 may 2026</t>
+          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -42584,7 +42584,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 02:24 · W20 · 12-18 may 2026</t>
+          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -42744,7 +42744,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 02:24 · W20 · 12-18 may 2026</t>
+          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -47342,7 +47342,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 02:24 · W20 · 12-18 may 2026</t>
+          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -47502,7 +47502,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 02:24 · W20 · 12-18 may 2026</t>
+          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -50981,7 +50981,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 02:24 · W20 · 12-18 may 2026</t>
+          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -55280,7 +55280,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 02:24 · W20 · 12-18 may 2026</t>
+          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -59579,7 +59579,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 02:24 · W20 · 12-18 may 2026</t>
+          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -61357,7 +61357,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 02:24 · W20 · 12-18 may 2026</t>
+          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -64951,7 +64951,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 02:24 · W20 · 12-18 may 2026</t>
+          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -65370,7 +65370,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 02:24 · W20 · 12-18 may 2026</t>
+          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -69669,7 +69669,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 02:24 · W20 · 12-18 may 2026</t>
+          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -73967,7 +73967,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 02:24 · W20 · 12-18 may 2026</t>
+          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -77961,7 +77961,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 02:24 · W20 · 12-18 may 2026</t>
+          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -80139,7 +80139,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 02:24 · W20 · 12-18 may 2026</t>
+          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -83733,7 +83733,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 02:24 · W20 · 12-18 may 2026</t>
+          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -84152,7 +84152,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 02:24 · W20 · 12-18 may 2026</t>
+          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Week 20 · RatesNoDispo + CheckRates + hub index · 11-17 may 2026 · WoW real W19
</commit_message>
<xml_diff>
--- a/checkrates/week-20/Analisis_Checkrates_7d.xlsx
+++ b/checkrates/week-20/Analisis_Checkrates_7d.xlsx
@@ -569,7 +569,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -725,7 +725,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1178,7 +1178,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1338,7 +1338,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1892,7 +1892,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -5099,7 +5099,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -9398,7 +9398,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -10736,7 +10736,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -14330,7 +14330,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -14669,7 +14669,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -18752,7 +18752,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -18905,7 +18905,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -19058,7 +19058,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -19218,7 +19218,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -23822,7 +23822,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -28121,7 +28121,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -32420,7 +32420,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -34278,7 +34278,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -37872,7 +37872,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -38291,7 +38291,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -42584,7 +42584,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -42744,7 +42744,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -47342,7 +47342,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -47502,7 +47502,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -50981,7 +50981,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -55280,7 +55280,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -59579,7 +59579,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -61357,7 +61357,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -64951,7 +64951,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -65370,7 +65370,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -69669,7 +69669,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -73967,7 +73967,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -77961,7 +77961,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -80139,7 +80139,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -83733,7 +83733,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -84152,7 +84152,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 23/05/2026 22:34 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Week 20 · RatesNoDispo + CheckRates + hub index · 11-17 may 2026
- Regeneración completa W20 con datasets W20/W19
- Sprint A: fixes visuales global vs canastas (headers tabs, wow pills, regex hist)
- Sprint B: centralización helpers (tab_column_header, make_wow_pill_row, wow_box compact)
- Fix searchbox canastas CR: panels tp-{card_id} con scope aislado
- Scripts actualizados: render_helpers, render_cr_p1/p3, render_rnd_p1/p3, asset heads
</commit_message>
<xml_diff>
--- a/checkrates/week-20/Analisis_Checkrates_7d.xlsx
+++ b/checkrates/week-20/Analisis_Checkrates_7d.xlsx
@@ -569,7 +569,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 21:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -725,7 +725,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 21:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 21:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1178,7 +1178,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 21:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1338,7 +1338,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 21:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -1892,7 +1892,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 21:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -5099,7 +5099,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 21:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -9398,7 +9398,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 21:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -10736,7 +10736,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 21:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -14330,7 +14330,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 21:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -14669,7 +14669,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 21:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -18752,7 +18752,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 21:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -18905,7 +18905,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 21:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -19058,7 +19058,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 21:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -19218,7 +19218,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 21:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -23822,7 +23822,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 21:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -28121,7 +28121,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 21:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -32420,7 +32420,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 21:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -34278,7 +34278,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 21:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -37872,7 +37872,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 21:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -38291,7 +38291,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 21:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -42584,7 +42584,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 21:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -42744,7 +42744,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 21:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -47342,7 +47342,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 21:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -47502,7 +47502,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 21:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -50981,7 +50981,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 21:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -55280,7 +55280,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 21:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -59579,7 +59579,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 21:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -61357,7 +61357,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 21:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -64951,7 +64951,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 21:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -65370,7 +65370,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 21:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -69669,7 +69669,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 21:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -73967,7 +73967,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 21:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -77961,7 +77961,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 21:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -80139,7 +80139,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 21:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -83733,7 +83733,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 21:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>
@@ -84152,7 +84152,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generado: 24/05/2026 03:40 · W20 · 12-18 may 2026</t>
+          <t>Generado: 24/05/2026 21:05 · W20 · 12-18 may 2026</t>
         </is>
       </c>
     </row>

</xml_diff>